<commit_message>
docs_api명세서 add, api_views_code update
</commit_message>
<xml_diff>
--- a/docs/요구사항_정의서.xlsx
+++ b/docs/요구사항_정의서.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\관리자\Desktop\이정수꺼\GitProject3\MyPerfume\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C92EA56C-1164-4099-9323-EEC017D60DDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17E1ACB7-A32D-472B-8DAB-B4EBDAAE93E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{4FDBCDF3-D99F-47F0-9850-97A29FCF3D98}"/>
   </bookViews>
@@ -93,9 +93,6 @@
     <t>생일/기념일/첫 만남/직장 등 선물 상황을 선택해 TPO에 맞는 향을 추천 받는다.</t>
   </si>
   <si>
-    <t>선물 대상 유형(연인/친구/가족 등)과 선물 상대의 성별을 선택할 수 있다.</t>
-  </si>
-  <si>
     <t>대상자가 싫어할 가능성이 높은 비선호 향조 취향을 선택해 선물 추천에서 제외할 수 있다.</t>
   </si>
   <si>
@@ -229,6 +226,10 @@
   </si>
   <si>
     <t>사용자가 선택한 여러 향수와 매칭도 점수를 한번에 제공한다.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>선물 대상 유형(연인/친구/가족 등)을 선택할 수 있다.</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -327,54 +328,42 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -714,19 +703,19 @@
   <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="29.1640625" style="7" customWidth="1"/>
-    <col min="2" max="2" width="30" style="7" customWidth="1"/>
-    <col min="3" max="3" width="51.5" style="7" customWidth="1"/>
+    <col min="1" max="1" width="29.1640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="30" style="3" customWidth="1"/>
+    <col min="3" max="3" width="51.5" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="4" t="s">
         <v>0</v>
       </c>
     </row>
@@ -734,39 +723,37 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
     </row>
     <row r="3" spans="1:4" ht="51" x14ac:dyDescent="0.45">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="8" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="34" x14ac:dyDescent="0.45">
-      <c r="A4" s="8"/>
-      <c r="B4" s="6"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="8"/>
       <c r="C4" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A5" s="8"/>
+      <c r="A5" s="11"/>
       <c r="B5" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="15"/>
+        <v>26</v>
+      </c>
+      <c r="D5" s="7"/>
     </row>
     <row r="6" spans="1:4" ht="61.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="8"/>
+      <c r="A6" s="11"/>
       <c r="B6" s="2" t="s">
         <v>8</v>
       </c>
@@ -775,242 +762,242 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="10" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A8" s="8"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
+      <c r="A8" s="11"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
     </row>
     <row r="9" spans="1:4" ht="34" x14ac:dyDescent="0.45">
-      <c r="A9" s="8"/>
+      <c r="A9" s="11"/>
       <c r="B9" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="65" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="11" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="65" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="8" t="s">
         <v>13</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="34" x14ac:dyDescent="0.45">
-      <c r="A12" s="8"/>
-      <c r="B12" s="3"/>
+      <c r="A12" s="11"/>
+      <c r="B12" s="8"/>
       <c r="C12" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A13" s="8"/>
+      <c r="A13" s="11"/>
       <c r="B13" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A14" s="8"/>
+      <c r="A14" s="11"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
     </row>
     <row r="15" spans="1:4" ht="34" x14ac:dyDescent="0.45">
-      <c r="A15" s="8"/>
-      <c r="B15" s="4" t="s">
+      <c r="A15" s="11"/>
+      <c r="B15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A16" s="11"/>
+      <c r="B16" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="34" x14ac:dyDescent="0.45">
-      <c r="A16" s="8"/>
-      <c r="B16" s="4" t="s">
+      <c r="C16" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="34" x14ac:dyDescent="0.45">
+      <c r="A17" s="11"/>
+      <c r="B17" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C17" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="34" x14ac:dyDescent="0.45">
-      <c r="A17" s="8"/>
-      <c r="B17" s="4" t="s">
+    <row r="18" spans="1:3" ht="34" x14ac:dyDescent="0.45">
+      <c r="A18" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="34" x14ac:dyDescent="0.45">
+      <c r="A19" s="11"/>
+      <c r="B19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="34" x14ac:dyDescent="0.45">
+      <c r="A20" s="11"/>
+      <c r="B20" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A21" s="11"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A22" s="11"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A23" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="34" x14ac:dyDescent="0.45">
-      <c r="A18" s="8" t="s">
+    </row>
+    <row r="24" spans="1:3" ht="51" x14ac:dyDescent="0.45">
+      <c r="A24" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="34" x14ac:dyDescent="0.45">
+      <c r="A25" s="9"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="34" x14ac:dyDescent="0.45">
-      <c r="A19" s="8"/>
-      <c r="B19" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="34" x14ac:dyDescent="0.45">
-      <c r="A20" s="8"/>
-      <c r="B20" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A21" s="8"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A22" s="8"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A23" s="7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="51" x14ac:dyDescent="0.45">
-      <c r="A24" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="34" x14ac:dyDescent="0.45">
-      <c r="A25" s="11"/>
-      <c r="B25" s="6"/>
-      <c r="C25" s="2" t="s">
-        <v>23</v>
-      </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A26" s="11"/>
+      <c r="A26" s="9"/>
       <c r="B26" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="C27" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A28" s="9"/>
+      <c r="B28" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C28" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A28" s="11"/>
-      <c r="B28" s="7" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A29" s="9"/>
+      <c r="B29" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C29" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A30" s="9" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A29" s="11"/>
-      <c r="B29" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A30" s="11" t="s">
+      <c r="B30" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="C30" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A31" s="9"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A32" s="9"/>
+      <c r="B32" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C32" s="2" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A31" s="11"/>
-      <c r="B31" s="9"/>
-      <c r="C31" s="9"/>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A32" s="11"/>
-      <c r="B32" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="A3:A6"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="A11:A17"/>
+    <mergeCell ref="A18:A22"/>
     <mergeCell ref="B24:B25"/>
     <mergeCell ref="A24:A26"/>
     <mergeCell ref="B30:B31"/>
     <mergeCell ref="C30:C31"/>
     <mergeCell ref="A27:A29"/>
     <mergeCell ref="A30:A32"/>
-    <mergeCell ref="B20:B22"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="A11:A17"/>
-    <mergeCell ref="A18:A22"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="A3:A6"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C13:C14"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>